<commit_message>
Rebuild Tech Products workbook without manual XML edits so it opens in Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgQYirZi3Bne6tXkabEbMs
</commit_message>
<xml_diff>
--- a/excel-basic-analytics/Technological-Products-Data.xlsx
+++ b/excel-basic-analytics/Technological-Products-Data.xlsx
@@ -12,28 +12,6 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -667,11 +645,11 @@
       </c>
       <c r="I4" s="9">
         <f>MIN(F2:F31)</f>
-        <v>229</v>
-      </c>
-      <c r="J4" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J4" s="10">
         <f>_xlfn.FORMULATEXT(I4)</f>
-        <v>=MIN(F2:F31)</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -708,11 +686,11 @@
       </c>
       <c r="I5" s="9">
         <f>MAX(F2:F31)</f>
-        <v>1999</v>
-      </c>
-      <c r="J5" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J5" s="10">
         <f>_xlfn.FORMULATEXT(I5)</f>
-        <v>=MAX(F2:F31)</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -749,11 +727,11 @@
       </c>
       <c r="I6" s="11">
         <f>AVERAGE(F2:F31)</f>
-        <v>1056</v>
-      </c>
-      <c r="J6" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J6" s="10">
         <f>_xlfn.FORMULATEXT(I6)</f>
-        <v>=AVERAGE(F2:F31)</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -853,11 +831,11 @@
       </c>
       <c r="I9" s="12">
         <f>MIN(E2:E31)</f>
-        <v>44034</v>
-      </c>
-      <c r="J9" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J9" s="10">
         <f>_xlfn.FORMULATEXT(I9)</f>
-        <v>=MIN(E2:E31)</v>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -894,11 +872,11 @@
       </c>
       <c r="I10" s="12">
         <f>MAX(E2:E31)</f>
-        <v>44495</v>
-      </c>
-      <c r="J10" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J10" s="10">
         <f>_xlfn.FORMULATEXT(I10)</f>
-        <v>=MAX(E2:E31)</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -996,13 +974,13 @@
           <t>Список брендів (I13:I22)</t>
         </is>
       </c>
-      <c r="I13" cm="1" s="13" t="str">
+      <c r="I13" s="13">
         <f t="array" ref="I13:I22">_xlfn.UNIQUE(A2:A31)</f>
-        <v>Apple</v>
-      </c>
-      <c r="J13" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J13" s="10">
         <f>_xlfn.FORMULATEXT(I13)</f>
-        <v>=UNIQUE(A2:A31)</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1032,9 +1010,7 @@
       <c r="F14" s="5" t="n">
         <v>649</v>
       </c>
-      <c r="I14" s="13" t="str">
-        <v>Samsung</v>
-      </c>
+      <c r="I14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1063,9 +1039,7 @@
       <c r="F15" s="5" t="n">
         <v>1299</v>
       </c>
-      <c r="I15" s="13" t="str">
-        <v>Google</v>
-      </c>
+      <c r="I15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1094,9 +1068,7 @@
       <c r="F16" s="5" t="n">
         <v>499</v>
       </c>
-      <c r="I16" s="13" t="str">
-        <v>Sony</v>
-      </c>
+      <c r="I16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1125,9 +1097,7 @@
       <c r="F17" s="5" t="n">
         <v>1999</v>
       </c>
-      <c r="I17" s="13" t="str">
-        <v>Microsoft</v>
-      </c>
+      <c r="I17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1156,9 +1126,7 @@
       <c r="F18" s="5" t="n">
         <v>749</v>
       </c>
-      <c r="I18" s="13" t="str">
-        <v>Dell</v>
-      </c>
+      <c r="I18" s="13" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1187,9 +1155,7 @@
       <c r="F19" s="5" t="n">
         <v>999</v>
       </c>
-      <c r="I19" s="13" t="str">
-        <v>HP</v>
-      </c>
+      <c r="I19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1218,9 +1184,7 @@
       <c r="F20" s="5" t="n">
         <v>799</v>
       </c>
-      <c r="I20" s="13" t="str">
-        <v>Lenovo</v>
-      </c>
+      <c r="I20" s="13" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1249,9 +1213,7 @@
       <c r="F21" s="5" t="n">
         <v>699</v>
       </c>
-      <c r="I21" s="13" t="str">
-        <v>Asus</v>
-      </c>
+      <c r="I21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1280,9 +1242,7 @@
       <c r="F22" s="5" t="n">
         <v>1099</v>
       </c>
-      <c r="I22" s="13" t="str">
-        <v>Acer</v>
-      </c>
+      <c r="I22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1381,11 +1341,11 @@
       </c>
       <c r="I25" s="13">
         <f>COUNTA(C2:C31)</f>
-        <v>30</v>
-      </c>
-      <c r="J25" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J25" s="10">
         <f>_xlfn.FORMULATEXT(I25)</f>
-        <v>=COUNTA(C2:C31)</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1483,13 +1443,13 @@
           <t>Кількість унікальних країн</t>
         </is>
       </c>
-      <c r="I28" cm="1" s="13">
+      <c r="I28" s="13">
         <f t="array" ref="I28">COUNTA(_xlfn.UNIQUE(D2:D31))</f>
-        <v>6</v>
-      </c>
-      <c r="J28" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J28" s="10">
         <f>_xlfn.FORMULATEXT(I28)</f>
-        <v>=COUNTA(UNIQUE(D2:D31))</v>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1524,13 +1484,13 @@
           <t>Чи вірно, що країн більше ніж 5?</t>
         </is>
       </c>
-      <c r="I29" s="13" t="b">
+      <c r="I29" s="13">
         <f>I28&gt;5</f>
-        <v>1</v>
-      </c>
-      <c r="J29" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J29" s="10">
         <f>_xlfn.FORMULATEXT(I29)</f>
-        <v>=I28&gt;5</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1565,13 +1525,13 @@
           <t>Список країн (I30:I35)</t>
         </is>
       </c>
-      <c r="I30" cm="1" s="13" t="str">
+      <c r="I30" s="13">
         <f t="array" ref="I30:I35">_xlfn.UNIQUE(D2:D31)</f>
-        <v>United States</v>
-      </c>
-      <c r="J30" s="10" t="str">
+        <v/>
+      </c>
+      <c r="J30" s="10">
         <f>_xlfn.FORMULATEXT(I30)</f>
-        <v>=UNIQUE(D2:D31)</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -1601,29 +1561,19 @@
       <c r="F31" s="5" t="n">
         <v>599</v>
       </c>
-      <c r="I31" s="13" t="str">
-        <v>South Korea</v>
-      </c>
+      <c r="I31" s="13" t="n"/>
     </row>
     <row r="32">
-      <c r="I32" s="13" t="str">
-        <v>Japan</v>
-      </c>
+      <c r="I32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="I33" s="13" t="str">
-        <v>China</v>
-      </c>
+      <c r="I33" s="13" t="n"/>
     </row>
     <row r="34">
-      <c r="I34" s="13" t="str">
-        <v>Taiwan</v>
-      </c>
+      <c r="I34" s="13" t="n"/>
     </row>
     <row r="35">
-      <c r="I35" s="13" t="str">
-        <v>Malaysia</v>
-      </c>
+      <c r="I35" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Count unique models in question 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgQYirZi3Bne6tXkabEbMs
</commit_message>
<xml_diff>
--- a/excel-basic-analytics/Technological-Products-Data.xlsx
+++ b/excel-basic-analytics/Technological-Products-Data.xlsx
@@ -1336,11 +1336,11 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Всього моделей (рядків з моделлю)</t>
+          <t>Кількість унікальних моделей</t>
         </is>
       </c>
       <c r="I25" s="13">
-        <f>COUNTA(C2:C31)</f>
+        <f t="array" ref="I25">COUNTA(_xlfn.UNIQUE(C2:C31))</f>
         <v/>
       </c>
       <c r="J25" s="10">
@@ -1374,6 +1374,19 @@
       </c>
       <c r="F26" s="5" t="n">
         <v>899</v>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Довідково: всього рядків з моделлю</t>
+        </is>
+      </c>
+      <c r="I26" s="13">
+        <f>COUNTA(C2:C31)</f>
+        <v/>
+      </c>
+      <c r="J26" s="10">
+        <f>_xlfn.FORMULATEXT(I26)</f>
+        <v/>
       </c>
     </row>
     <row r="27">

</xml_diff>